<commit_message>
Segundo Parcial 25 porcentajes asistencia
</commit_message>
<xml_diff>
--- a/grupos/4AEM - Estadisticos 20222.xlsx
+++ b/grupos/4AEM - Estadisticos 20222.xlsx
@@ -3710,7 +3710,7 @@
         <v>98</v>
       </c>
       <c r="N4">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="O4">
         <v>100</v>
@@ -3731,7 +3731,7 @@
         <v>98</v>
       </c>
       <c r="U4">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="V4">
         <v>100</v>
@@ -3778,7 +3778,7 @@
         <v>100</v>
       </c>
       <c r="N5">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O5">
         <v>100</v>
@@ -3799,7 +3799,7 @@
         <v>100</v>
       </c>
       <c r="U5">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V5">
         <v>100</v>
@@ -3846,7 +3846,7 @@
         <v>82.40000000000001</v>
       </c>
       <c r="N6">
-        <v>83.09999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="O6">
         <v>100</v>
@@ -3867,7 +3867,7 @@
         <v>82.40000000000001</v>
       </c>
       <c r="U6">
-        <v>83.09999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="V6">
         <v>100</v>
@@ -3914,7 +3914,7 @@
         <v>88.2</v>
       </c>
       <c r="N7">
-        <v>83.09999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="O7">
         <v>100</v>
@@ -3935,7 +3935,7 @@
         <v>88.2</v>
       </c>
       <c r="U7">
-        <v>83.09999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="V7">
         <v>100</v>
@@ -3982,7 +3982,7 @@
         <v>98</v>
       </c>
       <c r="N8">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="O8">
         <v>100</v>
@@ -4003,7 +4003,7 @@
         <v>98</v>
       </c>
       <c r="U8">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="V8">
         <v>100</v>
@@ -4050,7 +4050,7 @@
         <v>66.7</v>
       </c>
       <c r="N9">
-        <v>66.2</v>
+        <v>67.2</v>
       </c>
       <c r="O9">
         <v>38.3</v>
@@ -4071,7 +4071,7 @@
         <v>66.7</v>
       </c>
       <c r="U9">
-        <v>66.2</v>
+        <v>67.2</v>
       </c>
       <c r="V9">
         <v>38.3</v>
@@ -4118,7 +4118,7 @@
         <v>90.2</v>
       </c>
       <c r="N10">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O10">
         <v>100</v>
@@ -4139,7 +4139,7 @@
         <v>90.2</v>
       </c>
       <c r="U10">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V10">
         <v>100</v>
@@ -4186,7 +4186,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="N11">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O11">
         <v>100</v>
@@ -4207,7 +4207,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="U11">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V11">
         <v>100</v>
@@ -4254,7 +4254,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="N12">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O12">
         <v>91.7</v>
@@ -4275,7 +4275,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="U12">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V12">
         <v>91.7</v>
@@ -4322,7 +4322,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="N13">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="O13">
         <v>100</v>
@@ -4343,7 +4343,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="U13">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="V13">
         <v>100</v>
@@ -4390,7 +4390,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="N14">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="O14">
         <v>100</v>
@@ -4411,7 +4411,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="U14">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="V14">
         <v>100</v>
@@ -4458,7 +4458,7 @@
         <v>88.2</v>
       </c>
       <c r="N15">
-        <v>86.2</v>
+        <v>87.5</v>
       </c>
       <c r="O15">
         <v>88.3</v>
@@ -4479,7 +4479,7 @@
         <v>88.2</v>
       </c>
       <c r="U15">
-        <v>86.2</v>
+        <v>87.5</v>
       </c>
       <c r="V15">
         <v>88.3</v>
@@ -4526,7 +4526,7 @@
         <v>86.3</v>
       </c>
       <c r="N16">
-        <v>90.8</v>
+        <v>92.2</v>
       </c>
       <c r="O16">
         <v>88.3</v>
@@ -4547,7 +4547,7 @@
         <v>86.3</v>
       </c>
       <c r="U16">
-        <v>90.8</v>
+        <v>92.2</v>
       </c>
       <c r="V16">
         <v>88.3</v>
@@ -4594,7 +4594,7 @@
         <v>82.40000000000001</v>
       </c>
       <c r="N17">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O17">
         <v>100</v>
@@ -4615,7 +4615,7 @@
         <v>82.40000000000001</v>
       </c>
       <c r="U17">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V17">
         <v>100</v>
@@ -4662,7 +4662,7 @@
         <v>88.2</v>
       </c>
       <c r="N18">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O18">
         <v>100</v>
@@ -4683,7 +4683,7 @@
         <v>88.2</v>
       </c>
       <c r="U18">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V18">
         <v>100</v>
@@ -4730,7 +4730,7 @@
         <v>84.3</v>
       </c>
       <c r="N19">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="O19">
         <v>100</v>
@@ -4751,7 +4751,7 @@
         <v>84.3</v>
       </c>
       <c r="U19">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="V19">
         <v>100</v>
@@ -4798,7 +4798,7 @@
         <v>88.2</v>
       </c>
       <c r="N20">
-        <v>89.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="O20">
         <v>100</v>
@@ -4819,7 +4819,7 @@
         <v>88.2</v>
       </c>
       <c r="U20">
-        <v>89.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="V20">
         <v>100</v>
@@ -4866,7 +4866,7 @@
         <v>78.40000000000001</v>
       </c>
       <c r="N21">
-        <v>83.09999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="O21">
         <v>90</v>
@@ -4887,7 +4887,7 @@
         <v>78.40000000000001</v>
       </c>
       <c r="U21">
-        <v>83.09999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="V21">
         <v>90</v>
@@ -4934,7 +4934,7 @@
         <v>78.40000000000001</v>
       </c>
       <c r="N22">
-        <v>84.59999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="O22">
         <v>83.3</v>
@@ -4955,7 +4955,7 @@
         <v>78.40000000000001</v>
       </c>
       <c r="U22">
-        <v>84.59999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="V22">
         <v>83.3</v>
@@ -5002,7 +5002,7 @@
         <v>98</v>
       </c>
       <c r="N23">
-        <v>96.90000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="O23">
         <v>100</v>
@@ -5023,7 +5023,7 @@
         <v>98</v>
       </c>
       <c r="U23">
-        <v>96.90000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="V23">
         <v>100</v>
@@ -5070,7 +5070,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="N24">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="O24">
         <v>91.7</v>
@@ -5091,7 +5091,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="U24">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="V24">
         <v>91.7</v>
@@ -5138,7 +5138,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="N25">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O25">
         <v>100</v>
@@ -5159,7 +5159,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="U25">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V25">
         <v>100</v>
@@ -5206,7 +5206,7 @@
         <v>92.2</v>
       </c>
       <c r="N26">
-        <v>92.3</v>
+        <v>93.8</v>
       </c>
       <c r="O26">
         <v>93.3</v>
@@ -5227,7 +5227,7 @@
         <v>92.2</v>
       </c>
       <c r="U26">
-        <v>92.3</v>
+        <v>93.8</v>
       </c>
       <c r="V26">
         <v>93.3</v>
@@ -5274,7 +5274,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="N27">
-        <v>92.3</v>
+        <v>93.8</v>
       </c>
       <c r="O27">
         <v>93.3</v>
@@ -5295,7 +5295,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="U27">
-        <v>92.3</v>
+        <v>93.8</v>
       </c>
       <c r="V27">
         <v>93.3</v>
@@ -5342,7 +5342,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="N28">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O28">
         <v>100</v>
@@ -5363,7 +5363,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="U28">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V28">
         <v>100</v>
@@ -5410,7 +5410,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="N29">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O29">
         <v>100</v>
@@ -5431,7 +5431,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="U29">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V29">
         <v>100</v>
@@ -5478,7 +5478,7 @@
         <v>86.3</v>
       </c>
       <c r="N30">
-        <v>89.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="O30">
         <v>100</v>
@@ -5499,7 +5499,7 @@
         <v>86.3</v>
       </c>
       <c r="U30">
-        <v>89.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="V30">
         <v>100</v>
@@ -5546,7 +5546,7 @@
         <v>84.3</v>
       </c>
       <c r="N31">
-        <v>90.8</v>
+        <v>92.2</v>
       </c>
       <c r="O31">
         <v>100</v>
@@ -5567,7 +5567,7 @@
         <v>84.3</v>
       </c>
       <c r="U31">
-        <v>90.8</v>
+        <v>92.2</v>
       </c>
       <c r="V31">
         <v>100</v>
@@ -5614,7 +5614,7 @@
         <v>90.2</v>
       </c>
       <c r="N32">
-        <v>90.8</v>
+        <v>92.2</v>
       </c>
       <c r="O32">
         <v>100</v>
@@ -5635,7 +5635,7 @@
         <v>90.2</v>
       </c>
       <c r="U32">
-        <v>90.8</v>
+        <v>92.2</v>
       </c>
       <c r="V32">
         <v>100</v>
@@ -5682,7 +5682,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="N33">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="O33">
         <v>100</v>
@@ -5703,7 +5703,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="U33">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="V33">
         <v>100</v>
@@ -5750,7 +5750,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="N34">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O34">
         <v>100</v>
@@ -5771,7 +5771,7 @@
         <v>94.09999999999999</v>
       </c>
       <c r="U34">
-        <v>95.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="V34">
         <v>100</v>

</xml_diff>